<commit_message>
Refresh 17 MongolBank datasets (October 2026 update)
Through September 2026: total, individual, mortgage, SME and newly
issued loans, credit to the private sector, MNT and FX deposit rates,
MNT lending rate, M1, M2, bank balance sheet, USD/MNT monthly and
monthly major-currency rates. Daily exchange rates run to 28 Oct 2026,
and the 2026 year-to-date annual averages now cover Jan-Sep. External
debt adds Q2 2026. No revisions to previously published values.

International investment position already had Q2 2026; only
last_checked_at changed.

Excerpts that quote values are rewritten from the new CSVs in EN and MN
(e.g. M1's stale "over 11 trillion by 2026" claim, Q3 2026 new loans).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.mn/public/datasets/mongolbank-bank-balance-sheet.xlsx
+++ b/data.mn/public/datasets/mongolbank-bank-balance-sheet.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D272"/>
+  <dimension ref="A1:D274"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4779,6 +4779,38 @@
       </c>
       <c r="D272" t="n">
         <v>79538.70699999999</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B273" t="n">
+        <v>8967.593000000001</v>
+      </c>
+      <c r="C273" t="n">
+        <v>90620.315</v>
+      </c>
+      <c r="D273" t="n">
+        <v>81652.723</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B274" t="n">
+        <v>9138.621999999999</v>
+      </c>
+      <c r="C274" t="n">
+        <v>94937.473</v>
+      </c>
+      <c r="D274" t="n">
+        <v>85798.851</v>
       </c>
     </row>
   </sheetData>
@@ -4792,7 +4824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D272"/>
+  <dimension ref="A1:D274"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9159,6 +9191,38 @@
         <v>8776.029</v>
       </c>
     </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B273" t="n">
+        <v>90620.315</v>
+      </c>
+      <c r="C273" t="n">
+        <v>81652.723</v>
+      </c>
+      <c r="D273" t="n">
+        <v>8967.593000000001</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B274" t="n">
+        <v>94937.473</v>
+      </c>
+      <c r="C274" t="n">
+        <v>85798.851</v>
+      </c>
+      <c r="D274" t="n">
+        <v>9138.621999999999</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>